<commit_message>
docs: add multi-library serial workflow
</commit_message>
<xml_diff>
--- a/libs/porting-tasks-模板.xlsx
+++ b/libs/porting-tasks-模板.xlsx
@@ -1,223 +1,189 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19050" windowHeight="11070"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="19050" windowHeight="11070" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="移植任务" sheetId="1" r:id="rId1"/>
+    <sheet name="移植任务" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
-  <si>
-    <t>库名</t>
-  </si>
-  <si>
-    <t>Git 仓库</t>
-  </si>
-  <si>
-    <t>版本</t>
-  </si>
-  <si>
-    <t>状态</t>
-  </si>
-  <si>
-    <t>备注</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="21">
-    <font>
-      <sz val="11"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="22">
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
       <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <b val="1"/>
       <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
+      <b val="1"/>
+      <color theme="3"/>
       <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
       <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
+      <b val="1"/>
       <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
+      <b val="1"/>
       <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="34">
-    <fill>
-      <patternFill patternType="none"/>
+  <fills count="35">
+    <fill>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -412,6 +378,11 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004F81BD"/>
       </patternFill>
     </fill>
   </fills>
@@ -524,155 +495,158 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -727,12 +701,130 @@
     <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Codex</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>三方库名称</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>源码仓库地址</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>tag / branch / commit，可留空</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>多库模式下：否的库先执行，是的库后执行；不填默认是</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>需要审批的库先填待审批；审批后由 AI 回写通过/不通过；不需要审批的库写不需要审批</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>记录业务适配阶段结果</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>记录编译阶段结果</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>记录设备测试或 binary 测试结果</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>记录失败阶段、失败原因或补充说明</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1018,36 +1110,74 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="4"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
+    <row r="1" ht="38" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>库名</t>
+        </is>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Git 仓库</t>
+        </is>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>版本</t>
+        </is>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>是否需要用户审批方案（是/否，默认是）</t>
+        </is>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>审批结果（待审批/通过/不通过/不需要审批）</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>适配状态（待处理/pass/fail/skip）</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>编译状态（待处理/pass/fail/skip）</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>测试状态（待处理/pass/fail/skip）</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>失败原因/备注</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>